<commit_message>
docs(finanzas): incorporar validacion contable de mercado, retornos de socios Alvaro y Alan, y remover migracion akura y referencias
</commit_message>
<xml_diff>
--- a/Flujo de caja y financiamiento - TerraSense.xlsx
+++ b/Flujo de caja y financiamiento - TerraSense.xlsx
@@ -1373,7 +1373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:H52"/>
+  <dimension ref="B2:I63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="2" customWidth="1" style="77" min="1" max="1"/>
@@ -2292,6 +2292,274 @@
       <c r="B52" s="80" t="inlineStr">
         <is>
           <t>Se declara sin maquillarlo, igual que antes: a 5 años y a la tasa exigida del 20 % el VAN ahora es POSITIVO. Se revisaron tres supuestos que antes eran demasiado conservadores o estaban incompletos — 10 % de contingencia sobre la inversión, tasa real de la línea de corto plazo (15 % en vez de 23 %) y dotación de ensambladores dimensionada por horas de trabajo — sin tocar las tres condiciones de fondo del proyecto (sonda a precio real, sueldo de ambos socios desde el mes 1, techo de precio de $249.990). La argumentación completa está en la hoja TOMA DE DECISIONES.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>DISTRIBUCIÓN Y RETORNO FINANCIERO POR SOCIO FUNDADOR (50 % ÁLVARO / 50 % ALAN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>AÑO 0</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>AÑO 1</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>AÑO 2</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>AÑO 3</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>AÑO 4</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>AÑO 5</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>TOTAL 5 AÑOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Sueldo empresarial por socio (CLP/año)</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56">
+        <f>'GASTOS FIJOS 5 AÑOS'!C6/2</f>
+        <v/>
+      </c>
+      <c r="E56">
+        <f>'GASTOS FIJOS 5 AÑOS'!D6/2</f>
+        <v/>
+      </c>
+      <c r="F56">
+        <f>'GASTOS FIJOS 5 AÑOS'!E6/2</f>
+        <v/>
+      </c>
+      <c r="G56">
+        <f>'GASTOS FIJOS 5 AÑOS'!F6/2</f>
+        <v/>
+      </c>
+      <c r="H56">
+        <f>'GASTOS FIJOS 5 AÑOS'!G6/2</f>
+        <v/>
+      </c>
+      <c r="I56">
+        <f>SUM(D56:H56)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>→ Sueldo mensual bruto por socio</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57">
+        <f>D56/12</f>
+        <v/>
+      </c>
+      <c r="E57">
+        <f>E56/12</f>
+        <v/>
+      </c>
+      <c r="F57">
+        <f>F56/12</f>
+        <v/>
+      </c>
+      <c r="G57">
+        <f>G56/12</f>
+        <v/>
+      </c>
+      <c r="H57">
+        <f>H56/12</f>
+        <v/>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Flujo de fondos libre de caja de la empresa</t>
+        </is>
+      </c>
+      <c r="C58">
+        <f>C25</f>
+        <v/>
+      </c>
+      <c r="D58">
+        <f>D25</f>
+        <v/>
+      </c>
+      <c r="E58">
+        <f>E25</f>
+        <v/>
+      </c>
+      <c r="F58">
+        <f>F25</f>
+        <v/>
+      </c>
+      <c r="G58">
+        <f>G25</f>
+        <v/>
+      </c>
+      <c r="H58">
+        <f>H25</f>
+        <v/>
+      </c>
+      <c r="I58">
+        <f>SUM(D58:H58)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Reparto de dividendos por socio (50 % flujo libre)</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59">
+        <f>E58/2</f>
+        <v/>
+      </c>
+      <c r="F59">
+        <f>F58/2</f>
+        <v/>
+      </c>
+      <c r="G59">
+        <f>G58/2</f>
+        <v/>
+      </c>
+      <c r="H59">
+        <f>H58/2</f>
+        <v/>
+      </c>
+      <c r="I59">
+        <f>SUM(D59:H59)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>TOTAL INGRESOS POR SOCIO (Sueldo + Dividendos)</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60">
+        <f>D56+D59</f>
+        <v/>
+      </c>
+      <c r="E60">
+        <f>E56+E59</f>
+        <v/>
+      </c>
+      <c r="F60">
+        <f>F56+F59</f>
+        <v/>
+      </c>
+      <c r="G60">
+        <f>G56+G59</f>
+        <v/>
+      </c>
+      <c r="H60">
+        <f>H56+H59</f>
+        <v/>
+      </c>
+      <c r="I60">
+        <f>SUM(D60:H60)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>(−) Pie de capital inicial aportado por socio</t>
+        </is>
+      </c>
+      <c r="C61">
+        <f>-PARÁMETROS!C32/2</f>
+        <v/>
+      </c>
+      <c r="D61" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61">
+        <f>-PARÁMETROS!C32/2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>(=) RETORNO NETO EN EL BOLSILLO POR SOCIO</t>
+        </is>
+      </c>
+      <c r="I62">
+        <f>I60+I61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Nota explicativa: En el Año 1 el flujo libre de caja es negativo por la devolución íntegra de la línea de corto plazo ($5.000.000) y amortización del crédito bancario; ambos socios cubren sus costos de vida mediante su sueldo empresarial garantizado ($553.553/mes legal). Entre los Años 2 y 5, con el negocio generando excedentes de caja positivos, los socios retiran el 50 % del flujo libre cada uno en dividendos. A 5 años, cada socio acumula $51.042.636 en sueldos y $32.996.118 en dividendos, obteniendo un retorno total neto de +$79.588.754 CLP limpios tras recuperar íntegramente su pie de capital inicial de $4.450.000 (multiplicador de 17,9 veces el capital aportado).</t>
         </is>
       </c>
     </row>
@@ -7855,7 +8123,7 @@
       </c>
       <c r="H6" s="37" t="inlineStr">
         <is>
-          <t>Año 1 al IMM; sube a medida que el negocio lo sostiene</t>
+          <t>Sueldo empresarial (Art. 31 N° 6 LIR). Año 1: .553 c/u (IMM legal); Año 2: .000 c/u; Año 3: .000 c/u; Año 4: .000.000 c/u; Año 5: .200.000 c/u. Garantiza ingreso formal a Álvaro y Alan desde el mes 1 (.042.636 acumulados por socio a 5 años).</t>
         </is>
       </c>
     </row>
@@ -8018,7 +8286,7 @@
       </c>
       <c r="H12" s="37" t="inlineStr">
         <is>
-          <t>Escala con la dotación y con la formalización del taller</t>
+          <t>Outsourcing contable Pyme (Contabilizate, TuContador, ChileContador: 1,8 a 4,3 UF/mes = .000 a .000/mes para F29, Previred y Renta). Un contador interno indefinido costaría ,8M a ,2M/año (Robert Half / Indeed 2024-2026), inviable para 200 u/año (3-4 h/mes de trabajo real). Sube en Años 3-5 por patente municipal comercial del taller físico.</t>
         </is>
       </c>
     </row>

</xml_diff>